<commit_message>
Fix: + Đổi tên "Loại tàu" thành "Tên luồng hàng hải" tại Luồng hàng hải + Sửa lại dữ liệu dùng để tạo báo cáo Thống kê luồng hàng hải từ bảng gis_spatial_objects sang bảng luong_hang_hai + Sửa lại dữ liệu dùng để tạo báo cáo Thống kê vùng đón trả hoa tiêu, vùng quay trở tàu, ga tránh tàu, khu neo tránh trú bão từ bảng gis_spatial_objects sang bảng vung_nuoc + Sửa lỗi chính tả key của 2 Template Excel BCKCHT_166.xlsx và BCKCHT_167.xlsx
</commit_message>
<xml_diff>
--- a/src/main/resources/public/template_export/BCKCHT_166.xlsx
+++ b/src/main/resources/public/template_export/BCKCHT_166.xlsx
@@ -266,13 +266,13 @@
     <t>Cục Hàng hải và Đường thủy Việt Nam (Phòng KCHT)</t>
   </si>
   <si>
-    <t>${thiz.getCateOtherText('AUTH_ORG',table.value[0].donViQuanLyVanHanh.asText())}</t>
-  </si>
-  <si>
     <t>${idx+1}</t>
   </si>
   <si>
     <t>${table.value[0].ten.asText()}</t>
+  </si>
+  <si>
+    <t>${this.getCateOtherText('AUTH_ORG',table.value[0].donViQuanLyVanHanh.asText())}</t>
   </si>
 </sst>
 </file>
@@ -471,12 +471,21 @@
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -491,15 +500,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -789,12 +789,12 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R19"/>
-  <sheetFormatPr defaultRowHeight="12.75" ns2:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.85546875" style="1" customWidth="1"/>
     <col min="2" max="2" width="44.140625" style="1" customWidth="1"/>
@@ -807,49 +807,49 @@
     <col min="19" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ns2:dyDescent="0.2">
-      <c r="A1" s="24" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="25"/>
+      <c r="B1" s="28"/>
       <c r="C1" s="10"/>
       <c r="D1" s="10"/>
       <c r="E1" s="10"/>
       <c r="F1" s="10"/>
       <c r="K1" s="18"/>
       <c r="L1" s="18"/>
-      <c r="M1" s="24" t="s">
+      <c r="M1" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="N1" s="24"/>
-      <c r="O1" s="24"/>
-      <c r="P1" s="24"/>
-      <c r="Q1" s="24"/>
-      <c r="R1" s="24"/>
-    </row>
-    <row r="2" spans="1:18" ns2:dyDescent="0.2">
-      <c r="A2" s="25" t="s">
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="27"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="24"/>
+      <c r="B2" s="27"/>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
-      <c r="M2" s="25" t="s">
+      <c r="M2" s="28" t="s">
         <v>51</v>
       </c>
-      <c r="N2" s="25"/>
-      <c r="O2" s="25"/>
-      <c r="P2" s="25"/>
-      <c r="Q2" s="25"/>
-      <c r="R2" s="25"/>
-    </row>
-    <row r="3" spans="1:18" ht="12.75" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A3" s="25" t="s">
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="28"/>
+      <c r="Q2" s="28"/>
+      <c r="R2" s="28"/>
+    </row>
+    <row r="3" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="28" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="25"/>
+      <c r="B3" s="28"/>
       <c r="C3" s="10"/>
       <c r="D3" s="10"/>
       <c r="E3" s="10"/>
@@ -858,172 +858,172 @@
         <v>26</v>
       </c>
       <c r="L3" s="19"/>
-      <c r="M3" s="28" t="s">
+      <c r="M3" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28"/>
-      <c r="P3" s="28"/>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="28"/>
-    </row>
-    <row r="4" spans="1:18" ht="12.75" customHeight="1" ns2:dyDescent="0.2">
+      <c r="N3" s="31"/>
+      <c r="O3" s="31"/>
+      <c r="P3" s="31"/>
+      <c r="Q3" s="31"/>
+      <c r="R3" s="31"/>
+    </row>
+    <row r="4" spans="1:18" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="K4" s="20"/>
       <c r="L4" s="20"/>
-      <c r="M4" s="22" t="s">
+      <c r="M4" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-    </row>
-    <row r="5" spans="1:18" ht="15.75" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A5" s="26" t="s">
+      <c r="N4" s="26"/>
+      <c r="O4" s="26"/>
+      <c r="P4" s="26"/>
+      <c r="Q4" s="26"/>
+      <c r="R4" s="26"/>
+    </row>
+    <row r="5" spans="1:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="26"/>
-      <c r="C5" s="26"/>
-      <c r="D5" s="26"/>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
-      <c r="I5" s="26"/>
-      <c r="J5" s="26"/>
-      <c r="K5" s="26"/>
-      <c r="L5" s="26"/>
-      <c r="M5" s="26"/>
-      <c r="N5" s="26"/>
-      <c r="O5" s="26"/>
-      <c r="P5" s="26"/>
-    </row>
-    <row r="6" spans="1:18" ht="15.75" ns2:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
+      <c r="J5" s="29"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="29"/>
+      <c r="M5" s="29"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="29"/>
+      <c r="P5" s="29"/>
+    </row>
+    <row r="6" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-      <c r="G6" s="27"/>
-      <c r="H6" s="27"/>
-      <c r="I6" s="27"/>
-      <c r="J6" s="27"/>
-      <c r="K6" s="27"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="27"/>
-      <c r="N6" s="27"/>
-      <c r="O6" s="27"/>
-      <c r="P6" s="27"/>
-    </row>
-    <row r="8" spans="1:18" s="2" customFormat="1" ht="29.25" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A8" s="23" t="s">
+      <c r="B6" s="30"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="30"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="30"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="30"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="30"/>
+      <c r="K6" s="30"/>
+      <c r="L6" s="30"/>
+      <c r="M6" s="30"/>
+      <c r="N6" s="30"/>
+      <c r="O6" s="30"/>
+      <c r="P6" s="30"/>
+    </row>
+    <row r="8" spans="1:18" s="2" customFormat="1" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="25" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="23" t="s">
+      <c r="C8" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="23"/>
-      <c r="E8" s="23"/>
-      <c r="F8" s="23"/>
-      <c r="G8" s="23"/>
-      <c r="H8" s="23" t="s">
+      <c r="D8" s="25"/>
+      <c r="E8" s="25"/>
+      <c r="F8" s="25"/>
+      <c r="G8" s="25"/>
+      <c r="H8" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="I8" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="J8" s="23" t="s">
+      <c r="J8" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="23"/>
-      <c r="L8" s="23" t="s">
+      <c r="K8" s="25"/>
+      <c r="L8" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="M8" s="23"/>
-      <c r="N8" s="23"/>
-      <c r="O8" s="23"/>
-      <c r="P8" s="23"/>
-      <c r="Q8" s="29" t="s">
+      <c r="M8" s="25"/>
+      <c r="N8" s="25"/>
+      <c r="O8" s="25"/>
+      <c r="P8" s="25"/>
+      <c r="Q8" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="R8" s="29" t="s">
+      <c r="R8" s="22" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:18" s="2" customFormat="1" ht="21.75" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A9" s="23"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23" t="s">
+    <row r="9" spans="1:18" s="2" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="25"/>
+      <c r="B9" s="25"/>
+      <c r="C9" s="25" t="s">
         <v>14</v>
       </c>
-      <c r="D9" s="23" t="s">
+      <c r="D9" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="23"/>
-      <c r="F9" s="23" t="s">
+      <c r="E9" s="25"/>
+      <c r="F9" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="G9" s="23" t="s">
+      <c r="G9" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="23"/>
-      <c r="I9" s="23"/>
-      <c r="J9" s="23" t="s">
+      <c r="H9" s="25"/>
+      <c r="I9" s="25"/>
+      <c r="J9" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="K9" s="23" t="s">
+      <c r="K9" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="L9" s="23" t="s">
+      <c r="L9" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="M9" s="23" t="s">
+      <c r="M9" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="N9" s="23" t="s">
+      <c r="N9" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="O9" s="23" t="s">
+      <c r="O9" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="P9" s="23" t="s">
+      <c r="P9" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
-    </row>
-    <row r="10" spans="1:18" s="2" customFormat="1" ht="21.75" customHeight="1" ns2:dyDescent="0.2">
-      <c r="A10" s="23"/>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
+      <c r="Q9" s="23"/>
+      <c r="R9" s="23"/>
+    </row>
+    <row r="10" spans="1:18" s="2" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="25"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
       <c r="D10" s="11" t="s">
         <v>17</v>
       </c>
       <c r="E10" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
-      <c r="L10" s="23"/>
-      <c r="M10" s="23"/>
-      <c r="N10" s="23"/>
-      <c r="O10" s="23"/>
-      <c r="P10" s="23"/>
-      <c r="Q10" s="31"/>
-      <c r="R10" s="31"/>
-    </row>
-    <row r="11" spans="1:18" s="3" customFormat="1" ns2:dyDescent="0.2">
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="25"/>
+      <c r="I10" s="25"/>
+      <c r="J10" s="25"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="25"/>
+      <c r="M10" s="25"/>
+      <c r="N10" s="25"/>
+      <c r="O10" s="25"/>
+      <c r="P10" s="25"/>
+      <c r="Q10" s="24"/>
+      <c r="R10" s="24"/>
+    </row>
+    <row r="11" spans="1:18" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="17" t="s">
         <v>1</v>
       </c>
@@ -1079,12 +1079,12 @@
         <v>16</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="63" customHeight="1" ns2:dyDescent="0.2">
+    <row r="12" spans="1:18" ht="63" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>55</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>56</v>
       </c>
       <c r="C12" s="14" t="e">
         <f>SUMPRODUCT(VALUE(C13))</f>
@@ -1115,10 +1115,10 @@
       </c>
       <c r="Q12" s="8"/>
       <c r="R12" s="21" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="20.100000000000001" customHeight="1" ns2:dyDescent="0.2">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="6"/>
       <c r="B13" s="7" t="s">
         <v>34</v>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="R13" s="8"/>
     </row>
-    <row r="15" spans="1:18" ns2:dyDescent="0.2">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="33" t="s">
         <v>5</v>
       </c>
@@ -1179,7 +1179,7 @@
       <c r="O15" s="34"/>
       <c r="P15" s="34"/>
     </row>
-    <row r="16" spans="1:18" ns2:dyDescent="0.2">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="32" t="s">
         <v>6</v>
       </c>
@@ -1198,7 +1198,7 @@
       <c r="O16" s="32"/>
       <c r="P16" s="32"/>
     </row>
-    <row r="17" spans="1:16" ns2:dyDescent="0.2">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A17" s="32"/>
       <c r="B17" s="32"/>
       <c r="C17" s="12"/>
@@ -1213,7 +1213,7 @@
       <c r="O17" s="32"/>
       <c r="P17" s="32"/>
     </row>
-    <row r="18" spans="1:16" ns2:dyDescent="0.2">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A18" s="32"/>
       <c r="B18" s="32"/>
       <c r="C18" s="12"/>
@@ -1228,7 +1228,7 @@
       <c r="O18" s="32"/>
       <c r="P18" s="32"/>
     </row>
-    <row r="19" spans="1:16" ns2:dyDescent="0.2">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A19" s="32"/>
       <c r="B19" s="32"/>
       <c r="C19" s="12"/>
@@ -1245,10 +1245,6 @@
     </row>
   </sheetData>
   <mergeCells count="33">
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="O9:O10"/>
-    <mergeCell ref="C9:C10"/>
     <mergeCell ref="J16:P19"/>
     <mergeCell ref="A16:B19"/>
     <mergeCell ref="A15:B15"/>
@@ -1261,10 +1257,6 @@
     <mergeCell ref="L8:P8"/>
     <mergeCell ref="L9:L10"/>
     <mergeCell ref="M9:M10"/>
-    <mergeCell ref="N9:N10"/>
-    <mergeCell ref="M4:R4"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="P9:P10"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="J8:K8"/>
@@ -1277,10 +1269,18 @@
     <mergeCell ref="Q8:Q10"/>
     <mergeCell ref="B8:B10"/>
     <mergeCell ref="M2:R2"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="O9:O10"/>
+    <mergeCell ref="C9:C10"/>
     <mergeCell ref="R8:R10"/>
+    <mergeCell ref="N9:N10"/>
+    <mergeCell ref="M4:R4"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="P9:P10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="3" fitToWidth="1" fitToHeight="0" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="3" fitToHeight="0" orientation="landscape" r:id="rId1"/>
   <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>